<commit_message>
Fix Database Add LessonProgress, Add License AI Generate
</commit_message>
<xml_diff>
--- a/src/mocks/greenlight_data.xlsx
+++ b/src/mocks/greenlight_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SmartDrivingLearningSystem\smart_driving_learning_system\src\mocks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56494AA9-6D99-4E12-8D5C-0A7E66187A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9EFF6D-A3C2-4380-9999-DABE01780397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Role" sheetId="1" r:id="rId1"/>
@@ -26,39 +26,40 @@
     <sheet name="UserLicense" sheetId="39" r:id="rId11"/>
     <sheet name="QuestionChapter" sheetId="10" r:id="rId12"/>
     <sheet name="QuestionLesson" sheetId="11" r:id="rId13"/>
-    <sheet name="QuestionTopic" sheetId="37" r:id="rId14"/>
-    <sheet name="QuestionCategory" sheetId="38" r:id="rId15"/>
-    <sheet name="Question" sheetId="12" r:id="rId16"/>
-    <sheet name="Tag" sheetId="13" r:id="rId17"/>
-    <sheet name="QuestionTag" sheetId="14" r:id="rId18"/>
-    <sheet name="SavedQuestion" sheetId="15" r:id="rId19"/>
-    <sheet name="LearningProgress" sheetId="16" r:id="rId20"/>
-    <sheet name="Answer" sheetId="17" r:id="rId21"/>
-    <sheet name="Exam" sheetId="18" r:id="rId22"/>
-    <sheet name="ExamQuestion" sheetId="19" r:id="rId23"/>
-    <sheet name="ExamSession" sheetId="20" r:id="rId24"/>
-    <sheet name="ExamDetail" sheetId="21" r:id="rId25"/>
-    <sheet name="ForumTopic" sheetId="22" r:id="rId26"/>
-    <sheet name="ForumPost" sheetId="23" r:id="rId27"/>
-    <sheet name="PostImage" sheetId="24" r:id="rId28"/>
-    <sheet name="PostReact" sheetId="25" r:id="rId29"/>
-    <sheet name="ForumComment" sheetId="26" r:id="rId30"/>
-    <sheet name="CommentVote" sheetId="27" r:id="rId31"/>
-    <sheet name="SignCategory" sheetId="28" r:id="rId32"/>
-    <sheet name="TrafficSign" sheetId="29" r:id="rId33"/>
-    <sheet name="SavedTrafficSign" sheetId="30" r:id="rId34"/>
-    <sheet name="ReportCategory" sheetId="31" r:id="rId35"/>
-    <sheet name="Report" sheetId="32" r:id="rId36"/>
-    <sheet name="Resolve" sheetId="33" r:id="rId37"/>
-    <sheet name="Notification" sheetId="34" r:id="rId38"/>
-    <sheet name="UserNotification" sheetId="35" r:id="rId39"/>
+    <sheet name="LessonProgress" sheetId="40" r:id="rId14"/>
+    <sheet name="QuestionTopic" sheetId="37" r:id="rId15"/>
+    <sheet name="QuestionCategory" sheetId="38" r:id="rId16"/>
+    <sheet name="Question" sheetId="12" r:id="rId17"/>
+    <sheet name="Tag" sheetId="13" r:id="rId18"/>
+    <sheet name="QuestionTag" sheetId="14" r:id="rId19"/>
+    <sheet name="SavedQuestion" sheetId="15" r:id="rId20"/>
+    <sheet name="LearningProgress" sheetId="16" r:id="rId21"/>
+    <sheet name="Answer" sheetId="17" r:id="rId22"/>
+    <sheet name="Exam" sheetId="18" r:id="rId23"/>
+    <sheet name="ExamQuestion" sheetId="19" r:id="rId24"/>
+    <sheet name="ExamSession" sheetId="20" r:id="rId25"/>
+    <sheet name="ExamDetail" sheetId="21" r:id="rId26"/>
+    <sheet name="ForumTopic" sheetId="22" r:id="rId27"/>
+    <sheet name="ForumPost" sheetId="23" r:id="rId28"/>
+    <sheet name="PostImage" sheetId="24" r:id="rId29"/>
+    <sheet name="PostReact" sheetId="25" r:id="rId30"/>
+    <sheet name="ForumComment" sheetId="26" r:id="rId31"/>
+    <sheet name="CommentVote" sheetId="27" r:id="rId32"/>
+    <sheet name="SignCategory" sheetId="28" r:id="rId33"/>
+    <sheet name="TrafficSign" sheetId="29" r:id="rId34"/>
+    <sheet name="SavedTrafficSign" sheetId="30" r:id="rId35"/>
+    <sheet name="ReportCategory" sheetId="31" r:id="rId36"/>
+    <sheet name="Report" sheetId="32" r:id="rId37"/>
+    <sheet name="Resolve" sheetId="33" r:id="rId38"/>
+    <sheet name="Notification" sheetId="34" r:id="rId39"/>
+    <sheet name="UserNotification" sheetId="35" r:id="rId40"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10115" uniqueCount="2976">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10125" uniqueCount="2976">
   <si>
     <t>id</t>
   </si>
@@ -9793,6 +9794,83 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2F0C51F-F730-40D6-A3D2-B5A208EEA456}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{528F0255-D674-42A9-8860-2BF5CD404E12}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9870,7 +9948,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38B320CB-917C-46B8-96F4-A2E982D167ED}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9948,7 +10026,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:L601"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -26560,7 +26638,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -26648,7 +26726,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -26709,82 +26787,6 @@
       </c>
       <c r="C3">
         <v>2</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>2946</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2946</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>2946</v>
@@ -27051,6 +27053,82 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -27127,7 +27205,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:G1859"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -69902,7 +69980,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70018,7 +70096,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70095,7 +70173,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70192,7 +70270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70269,7 +70347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70346,7 +70424,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70463,7 +70541,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70534,93 +70612,6 @@
       </c>
       <c r="D3" t="s">
         <v>80</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2946</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2942</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>2946</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3" t="s">
-        <v>2943</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>2946</v>
@@ -70746,6 +70737,93 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2942</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2943</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70839,7 +70917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70916,7 +70994,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -70993,7 +71071,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -71106,7 +71184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -71183,7 +71261,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -71260,7 +71338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -71383,7 +71461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -71480,7 +71558,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -71559,83 +71637,6 @@
         <v>2947</v>
       </c>
       <c r="G3">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2946</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>2946</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2947</v>
-      </c>
-      <c r="F3">
         <v>1</v>
       </c>
     </row>
@@ -71797,6 +71798,83 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2946</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2947</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>